<commit_message>
renaming dir from caregiver_client → from fall_dashboard
</commit_message>
<xml_diff>
--- a/_concept_6G_integration/MCS_Fall_Detection.xlsx
+++ b/_concept_6G_integration/MCS_Fall_Detection.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hayat\Documents\6G\FallDetection_new\_concept_6G_integration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31BC606B-2BFB-4C51-8CFF-EE3FC3843CB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D28CDA26-6BD0-468B-AFD5-B1AD770E0064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20544" yWindow="-2970" windowWidth="23232" windowHeight="13872" activeTab="2" xr2:uid="{55F2A534-9267-4FFE-9D89-C2FA8C43E60F}"/>
+    <workbookView xWindow="20544" yWindow="-2970" windowWidth="23232" windowHeight="13872" activeTab="3" xr2:uid="{55F2A534-9267-4FFE-9D89-C2FA8C43E60F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -675,12 +675,12 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4937,15 +4937,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>405541</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>35411</xdr:rowOff>
+      <xdr:colOff>232634</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>57824</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>217618</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>111611</xdr:rowOff>
+      <xdr:colOff>44711</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>134023</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -4960,8 +4960,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5282341" y="6344771"/>
-          <a:ext cx="1031277" cy="647700"/>
+          <a:off x="5109434" y="6324153"/>
+          <a:ext cx="1031277" cy="654423"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5002,18 +5002,18 @@
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
             </a:rPr>
-            <a:t>Grafana &amp; Prometeheus</a:t>
+            <a:t>Grafana </a:t>
           </a:r>
         </a:p>
         <a:p>
           <a:pPr algn="ctr"/>
           <a:r>
-            <a:rPr lang="en-GB" sz="900" baseline="0">
+            <a:rPr lang="en-GB" sz="1200" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
             </a:rPr>
-            <a:t>(Ml performance)</a:t>
+            <a:t>:3000</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -5116,6 +5116,17 @@
               </a:solidFill>
             </a:rPr>
             <a:t>)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>:5432</a:t>
           </a:r>
           <a:endParaRPr lang="en-DE" sz="1100">
             <a:solidFill>
@@ -5196,6 +5207,17 @@
               </a:solidFill>
             </a:rPr>
             <a:t>MLFlow</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1200">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>:5000</a:t>
           </a:r>
           <a:endParaRPr lang="en-DE" sz="1200">
             <a:solidFill>
@@ -5546,7 +5568,18 @@
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
             </a:rPr>
-            <a:t>API</a:t>
+            <a:t>API server</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1200">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>:8001</a:t>
           </a:r>
           <a:endParaRPr lang="en-DE" sz="1200">
             <a:solidFill>
@@ -5636,6 +5669,17 @@
             </a:rPr>
             <a:t> Broker</a:t>
           </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>:1883</a:t>
+          </a:r>
           <a:endParaRPr lang="en-DE" sz="1200">
             <a:solidFill>
               <a:schemeClr val="bg1"/>
@@ -5648,16 +5692,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>19691</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>94866</xdr:rowOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>185539</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>25053</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>444506</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>171066</xdr:rowOff>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>4564</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>101253</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -5672,8 +5716,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4896491" y="4415854"/>
-          <a:ext cx="1034415" cy="654424"/>
+          <a:off x="14815939" y="9953465"/>
+          <a:ext cx="1038225" cy="654423"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6925,6 +6969,21 @@
             </a:rPr>
             <a:t>Dashboard backend</a:t>
           </a:r>
+          <a:br>
+            <a:rPr lang="en-GB" sz="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>:8002</a:t>
+          </a:r>
           <a:endParaRPr lang="en-GB" sz="800" baseline="0">
             <a:solidFill>
               <a:schemeClr val="bg1"/>
@@ -7350,11 +7409,108 @@
             </a:rPr>
             <a:t>)</a:t>
           </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>:5432</a:t>
+          </a:r>
           <a:endParaRPr lang="en-DE" sz="1100">
             <a:solidFill>
               <a:schemeClr val="bg1"/>
             </a:solidFill>
           </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>214704</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>84717</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>32496</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>160916</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="77" name="Rectangle 76">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5E6DD959-4E17-4FCC-B702-14DE2252E107}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5091504" y="7122011"/>
+          <a:ext cx="1036992" cy="654423"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="002060"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:srgbClr val="002060"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Prometeheus</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>:9090</a:t>
+          </a:r>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -7822,7 +7978,7 @@
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
             </a:rPr>
-            <a:t>Caregiver</a:t>
+            <a:t>Fall</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-GB" sz="1000" baseline="0">
@@ -17871,19 +18027,19 @@
     </row>
     <row r="6" spans="18:35" ht="18.75" x14ac:dyDescent="0.3">
       <c r="X6" s="8"/>
-      <c r="Y6" s="25" t="s">
+      <c r="Y6" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="Z6" s="25"/>
-      <c r="AA6" s="25" t="s">
+      <c r="Z6" s="29"/>
+      <c r="AA6" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="AB6" s="25"/>
-      <c r="AC6" s="25"/>
-      <c r="AD6" s="26"/>
-      <c r="AE6" s="26"/>
-      <c r="AF6" s="26"/>
-      <c r="AG6" s="28" t="s">
+      <c r="AB6" s="29"/>
+      <c r="AC6" s="29"/>
+      <c r="AD6" s="25"/>
+      <c r="AE6" s="25"/>
+      <c r="AF6" s="25"/>
+      <c r="AG6" s="27" t="s">
         <v>91</v>
       </c>
       <c r="AH6" s="16"/>
@@ -17891,15 +18047,15 @@
     </row>
     <row r="7" spans="18:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="X7" s="8"/>
-      <c r="Y7" s="27"/>
-      <c r="Z7" s="27"/>
-      <c r="AA7" s="27"/>
-      <c r="AB7" s="27"/>
-      <c r="AC7" s="27"/>
-      <c r="AD7" s="27"/>
-      <c r="AE7" s="27"/>
-      <c r="AF7" s="27"/>
-      <c r="AG7" s="27"/>
+      <c r="Y7" s="26"/>
+      <c r="Z7" s="26"/>
+      <c r="AA7" s="26"/>
+      <c r="AB7" s="26"/>
+      <c r="AC7" s="26"/>
+      <c r="AD7" s="26"/>
+      <c r="AE7" s="26"/>
+      <c r="AF7" s="26"/>
+      <c r="AG7" s="26"/>
       <c r="AH7" s="8"/>
       <c r="AI7" s="8"/>
     </row>
@@ -18056,7 +18212,7 @@
       <c r="AD16" s="8"/>
       <c r="AE16" s="8"/>
       <c r="AF16" s="8"/>
-      <c r="AG16" s="29" t="s">
+      <c r="AG16" s="28" t="s">
         <v>96</v>
       </c>
       <c r="AH16" s="8"/>
@@ -18074,7 +18230,7 @@
       <c r="AD17" s="8"/>
       <c r="AE17" s="8"/>
       <c r="AF17" s="8"/>
-      <c r="AG17" s="29" t="s">
+      <c r="AG17" s="28" t="s">
         <v>95</v>
       </c>
       <c r="AH17" s="8"/>
@@ -18092,7 +18248,7 @@
       <c r="AD18" s="8"/>
       <c r="AE18" s="8"/>
       <c r="AF18" s="8"/>
-      <c r="AG18" s="29" t="s">
+      <c r="AG18" s="28" t="s">
         <v>95</v>
       </c>
       <c r="AH18" s="8"/>
@@ -18244,7 +18400,7 @@
       <c r="AD28" s="8"/>
       <c r="AE28" s="8"/>
       <c r="AF28" s="8"/>
-      <c r="AG28" s="29" t="s">
+      <c r="AG28" s="28" t="s">
         <v>99</v>
       </c>
       <c r="AH28" s="8"/>
@@ -18262,7 +18418,7 @@
       <c r="AD29" s="8"/>
       <c r="AE29" s="8"/>
       <c r="AF29" s="8"/>
-      <c r="AG29" s="29" t="s">
+      <c r="AG29" s="28" t="s">
         <v>99</v>
       </c>
       <c r="AH29" s="8"/>
@@ -18280,7 +18436,7 @@
       <c r="AD30" s="8"/>
       <c r="AE30" s="8"/>
       <c r="AF30" s="8"/>
-      <c r="AG30" s="29" t="s">
+      <c r="AG30" s="28" t="s">
         <v>99</v>
       </c>
       <c r="AH30" s="8"/>
@@ -18298,7 +18454,7 @@
       <c r="AD31" s="8"/>
       <c r="AE31" s="8"/>
       <c r="AF31" s="8"/>
-      <c r="AG31" s="29" t="s">
+      <c r="AG31" s="28" t="s">
         <v>99</v>
       </c>
       <c r="AH31" s="8"/>
@@ -18316,7 +18472,7 @@
       <c r="AD32" s="8"/>
       <c r="AE32" s="8"/>
       <c r="AF32" s="8"/>
-      <c r="AG32" s="29" t="s">
+      <c r="AG32" s="28" t="s">
         <v>99</v>
       </c>
       <c r="AH32" s="8"/>

</xml_diff>

<commit_message>
Refactor deployment architecture documentation to clarify InfluxDB's role, update ISA integration guide for mock server path, remove outdated MLflow retraining guide, and introduce MLOps retraining cycle documentation. Enhance inference server model switching functionality to support MLflow registry integration and add PowerShell script for model switching. Update retrain script to log artifacts correctly and modify model files accordingly.
</commit_message>
<xml_diff>
--- a/_concept_6G_integration/MCS_Fall_Detection.xlsx
+++ b/_concept_6G_integration/MCS_Fall_Detection.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hayat\Documents\6G\FallDetection_new\_concept_6G_integration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFE1DE29-E6B3-469E-8F3F-5AE37890C4DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCA650CF-BBE3-4C6E-9889-3B62ACDAAACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20544" yWindow="-2970" windowWidth="23232" windowHeight="13872" activeTab="2" xr2:uid="{55F2A534-9267-4FFE-9D89-C2FA8C43E60F}"/>
+    <workbookView xWindow="20544" yWindow="-2970" windowWidth="23232" windowHeight="13872" activeTab="3" xr2:uid="{55F2A534-9267-4FFE-9D89-C2FA8C43E60F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -4894,14 +4894,14 @@
     <xdr:from>
       <xdr:col>16</xdr:col>
       <xdr:colOff>436583</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>167096</xdr:rowOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>5442</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
       <xdr:colOff>168330</xdr:colOff>
       <xdr:row>29</xdr:row>
-      <xdr:rowOff>108857</xdr:rowOff>
+      <xdr:rowOff>110761</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -4916,8 +4916,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10190183" y="4662896"/>
-          <a:ext cx="1560547" cy="1465761"/>
+          <a:off x="10190183" y="4882242"/>
+          <a:ext cx="1560547" cy="1248319"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6464,14 +6464,14 @@
     <xdr:from>
       <xdr:col>9</xdr:col>
       <xdr:colOff>20732</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>76199</xdr:rowOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>445658</xdr:colOff>
+      <xdr:colOff>447563</xdr:colOff>
       <xdr:row>39</xdr:row>
-      <xdr:rowOff>28798</xdr:rowOff>
+      <xdr:rowOff>30703</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -6486,8 +6486,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5507132" y="4762499"/>
-          <a:ext cx="1644126" cy="3191099"/>
+          <a:off x="5507132" y="4648200"/>
+          <a:ext cx="1646031" cy="3307303"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6625,15 +6625,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>260488</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>183105</xdr:rowOff>
+      <xdr:colOff>269742</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>50843</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>276561</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>144124</xdr:rowOff>
+      <xdr:colOff>285815</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>11862</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -6648,8 +6648,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5746888" y="5100246"/>
-          <a:ext cx="1235273" cy="731984"/>
+          <a:off x="5756142" y="5499143"/>
+          <a:ext cx="1235273" cy="723019"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6726,16 +6726,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>104183</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>189810</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>340131</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>70067</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>523283</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>75511</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>149631</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>146268</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -6750,7 +6750,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10467383" y="5447610"/>
+          <a:off x="5826531" y="4756367"/>
           <a:ext cx="1028700" cy="647701"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6826,15 +6826,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>131285</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>26142</xdr:rowOff>
+      <xdr:colOff>98628</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>55262</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
-      <xdr:colOff>550385</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>104583</xdr:rowOff>
+      <xdr:colOff>517728</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>133703</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -6849,7 +6849,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10494485" y="4712442"/>
+          <a:off x="10461828" y="5122562"/>
           <a:ext cx="1028700" cy="649941"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6925,15 +6925,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>350086</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>125384</xdr:rowOff>
+      <xdr:colOff>166934</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>67418</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>145226</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>571674</xdr:colOff>
       <xdr:row>38</xdr:row>
-      <xdr:rowOff>5715</xdr:rowOff>
+      <xdr:rowOff>138249</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -6948,8 +6948,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5836486" y="6969937"/>
-          <a:ext cx="1014340" cy="844037"/>
+          <a:off x="5653334" y="7039718"/>
+          <a:ext cx="1014340" cy="832831"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -7456,15 +7456,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>227156</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>20944</xdr:rowOff>
+      <xdr:colOff>270700</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>91701</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>260536</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>78722</xdr:rowOff>
+      <xdr:colOff>307890</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>149479</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -7479,8 +7479,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5713556" y="6094532"/>
-          <a:ext cx="1252580" cy="636002"/>
+          <a:off x="5757100" y="6302001"/>
+          <a:ext cx="1256390" cy="629278"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -7973,13 +7973,13 @@
     <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>499141</xdr:colOff>
-      <xdr:row>114</xdr:row>
+      <xdr:row>115</xdr:row>
       <xdr:rowOff>66482</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>23</xdr:col>
       <xdr:colOff>321704</xdr:colOff>
-      <xdr:row>117</xdr:row>
+      <xdr:row>118</xdr:row>
       <xdr:rowOff>46196</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -11213,7 +11213,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Task (writer)</a:t>
+            <a:t>Task </a:t>
           </a:r>
           <a:endParaRPr lang="en-DE" sz="900">
             <a:effectLst/>
@@ -11391,7 +11391,7 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>142874</xdr:colOff>
+      <xdr:colOff>144779</xdr:colOff>
       <xdr:row>60</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:from>
@@ -11414,7 +11414,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="754379" y="304800"/>
+          <a:off x="754379" y="11544300"/>
           <a:ext cx="6694171" cy="327660"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -11451,15 +11451,7 @@
                 <a:schemeClr val="tx1"/>
               </a:solidFill>
             </a:rPr>
-            <a:t>Fall History Dashboard (needs</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-GB" sz="2000" b="1" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t> update)</a:t>
+            <a:t>Fall History Dashboard </a:t>
           </a:r>
           <a:endParaRPr lang="en-DE" sz="2000" b="1">
             <a:solidFill>
@@ -11767,13 +11759,13 @@
     <xdr:from>
       <xdr:col>21</xdr:col>
       <xdr:colOff>56606</xdr:colOff>
-      <xdr:row>97</xdr:row>
+      <xdr:row>98</xdr:row>
       <xdr:rowOff>117437</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
       <xdr:colOff>569868</xdr:colOff>
-      <xdr:row>97</xdr:row>
+      <xdr:row>98</xdr:row>
       <xdr:rowOff>117437</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -11831,14 +11823,14 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>27</xdr:col>
-      <xdr:colOff>38373</xdr:colOff>
-      <xdr:row>100</xdr:row>
+      <xdr:colOff>327212</xdr:colOff>
+      <xdr:row>101</xdr:row>
       <xdr:rowOff>150189</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>100</xdr:row>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>555812</xdr:colOff>
+      <xdr:row>101</xdr:row>
       <xdr:rowOff>150189</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -11854,8 +11846,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="16497573" y="19200189"/>
-          <a:ext cx="1790427" cy="0"/>
+          <a:off x="16786412" y="19424307"/>
+          <a:ext cx="1447800" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -12056,11 +12048,37 @@
           <a:r>
             <a:rPr lang="en-GB" sz="900" b="0">
               <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Backend</a:t>
-          </a:r>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="85000"/>
+                  <a:lumOff val="15000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Backend </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="85000"/>
+                  <a:lumOff val="15000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Compnents / System</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-GB" sz="900" b="0">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="85000"/>
+                <a:lumOff val="15000"/>
+              </a:schemeClr>
+            </a:solidFill>
+          </a:endParaRPr>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -12240,7 +12258,7 @@
                 <a:schemeClr val="tx1"/>
               </a:solidFill>
             </a:rPr>
-            <a:t> App</a:t>
+            <a:t> App Compnents / System</a:t>
           </a:r>
           <a:endParaRPr lang="en-GB" sz="900" b="0">
             <a:solidFill>
@@ -12321,13 +12339,13 @@
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>49529</xdr:colOff>
-      <xdr:row>94</xdr:row>
+      <xdr:row>95</xdr:row>
       <xdr:rowOff>96066</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>511629</xdr:colOff>
-      <xdr:row>94</xdr:row>
+      <xdr:row>95</xdr:row>
       <xdr:rowOff>96066</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -12462,15 +12480,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>60688</xdr:colOff>
-      <xdr:row>96</xdr:row>
-      <xdr:rowOff>63489</xdr:rowOff>
+      <xdr:colOff>49147</xdr:colOff>
+      <xdr:row>97</xdr:row>
+      <xdr:rowOff>90942</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>1905</xdr:colOff>
-      <xdr:row>98</xdr:row>
-      <xdr:rowOff>120540</xdr:rowOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>599964</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>147993</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -12485,8 +12503,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13471888" y="19113489"/>
-          <a:ext cx="550817" cy="438051"/>
+          <a:off x="13460347" y="18594095"/>
+          <a:ext cx="550817" cy="442533"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -12641,13 +12659,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>161652</xdr:colOff>
-      <xdr:row>88</xdr:row>
+      <xdr:row>89</xdr:row>
       <xdr:rowOff>134981</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>560614</xdr:colOff>
-      <xdr:row>88</xdr:row>
+      <xdr:row>89</xdr:row>
       <xdr:rowOff>134981</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -12706,13 +12724,13 @@
     <xdr:from>
       <xdr:col>23</xdr:col>
       <xdr:colOff>67764</xdr:colOff>
-      <xdr:row>97</xdr:row>
+      <xdr:row>98</xdr:row>
       <xdr:rowOff>119342</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>23</xdr:col>
       <xdr:colOff>575311</xdr:colOff>
-      <xdr:row>97</xdr:row>
+      <xdr:row>98</xdr:row>
       <xdr:rowOff>119342</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -12771,13 +12789,13 @@
     <xdr:from>
       <xdr:col>18</xdr:col>
       <xdr:colOff>189140</xdr:colOff>
-      <xdr:row>94</xdr:row>
+      <xdr:row>95</xdr:row>
       <xdr:rowOff>87902</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>20</xdr:col>
       <xdr:colOff>512718</xdr:colOff>
-      <xdr:row>94</xdr:row>
+      <xdr:row>95</xdr:row>
       <xdr:rowOff>87902</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -13099,15 +13117,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>164519</xdr:colOff>
-      <xdr:row>86</xdr:row>
-      <xdr:rowOff>167639</xdr:rowOff>
+      <xdr:colOff>166424</xdr:colOff>
+      <xdr:row>87</xdr:row>
+      <xdr:rowOff>130629</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>555812</xdr:colOff>
-      <xdr:row>88</xdr:row>
-      <xdr:rowOff>70965</xdr:rowOff>
+      <xdr:row>89</xdr:row>
+      <xdr:rowOff>72870</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -13122,8 +13140,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1993319" y="17321604"/>
-          <a:ext cx="8925693" cy="288808"/>
+          <a:off x="1995224" y="16704129"/>
+          <a:ext cx="8923788" cy="323241"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -13333,13 +13351,13 @@
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>51236</xdr:colOff>
-      <xdr:row>91</xdr:row>
+      <xdr:row>92</xdr:row>
       <xdr:rowOff>31024</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>566057</xdr:colOff>
-      <xdr:row>94</xdr:row>
+      <xdr:row>95</xdr:row>
       <xdr:rowOff>14548</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -13552,13 +13570,13 @@
     <xdr:from>
       <xdr:col>15</xdr:col>
       <xdr:colOff>450124</xdr:colOff>
-      <xdr:row>90</xdr:row>
+      <xdr:row>91</xdr:row>
       <xdr:rowOff>20138</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>20</xdr:col>
       <xdr:colOff>117455</xdr:colOff>
-      <xdr:row>91</xdr:row>
+      <xdr:row>92</xdr:row>
       <xdr:rowOff>140278</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -13725,15 +13743,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>118655</xdr:colOff>
+      <xdr:colOff>151312</xdr:colOff>
       <xdr:row>85</xdr:row>
-      <xdr:rowOff>86268</xdr:rowOff>
+      <xdr:rowOff>160835</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>442233</xdr:colOff>
+      <xdr:colOff>474890</xdr:colOff>
       <xdr:row>85</xdr:row>
-      <xdr:rowOff>86268</xdr:rowOff>
+      <xdr:rowOff>160835</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -13748,7 +13766,7 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7433855" y="16278768"/>
+          <a:off x="7466512" y="16353335"/>
           <a:ext cx="1542778" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
@@ -13791,13 +13809,13 @@
     <xdr:from>
       <xdr:col>24</xdr:col>
       <xdr:colOff>107225</xdr:colOff>
-      <xdr:row>93</xdr:row>
+      <xdr:row>94</xdr:row>
       <xdr:rowOff>111306</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>26</xdr:col>
       <xdr:colOff>582386</xdr:colOff>
-      <xdr:row>96</xdr:row>
+      <xdr:row>97</xdr:row>
       <xdr:rowOff>85453</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -13921,13 +13939,13 @@
     <xdr:from>
       <xdr:col>15</xdr:col>
       <xdr:colOff>52524</xdr:colOff>
-      <xdr:row>105</xdr:row>
+      <xdr:row>106</xdr:row>
       <xdr:rowOff>11221</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>26</xdr:col>
       <xdr:colOff>566681</xdr:colOff>
-      <xdr:row>105</xdr:row>
+      <xdr:row>106</xdr:row>
       <xdr:rowOff>11221</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -13986,13 +14004,13 @@
     <xdr:from>
       <xdr:col>24</xdr:col>
       <xdr:colOff>91440</xdr:colOff>
-      <xdr:row>97</xdr:row>
+      <xdr:row>98</xdr:row>
       <xdr:rowOff>128803</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>27</xdr:col>
       <xdr:colOff>5443</xdr:colOff>
-      <xdr:row>97</xdr:row>
+      <xdr:row>98</xdr:row>
       <xdr:rowOff>128803</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -14221,7 +14239,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Task (writer + trigerer)</a:t>
+            <a:t>Task </a:t>
           </a:r>
           <a:endParaRPr lang="en-DE" sz="900">
             <a:effectLst/>
@@ -14235,13 +14253,13 @@
     <xdr:from>
       <xdr:col>15</xdr:col>
       <xdr:colOff>171577</xdr:colOff>
-      <xdr:row>103</xdr:row>
+      <xdr:row>104</xdr:row>
       <xdr:rowOff>88351</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>26</xdr:col>
       <xdr:colOff>416186</xdr:colOff>
-      <xdr:row>104</xdr:row>
+      <xdr:row>105</xdr:row>
       <xdr:rowOff>150523</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -14378,6 +14396,219 @@
                 <a:lumOff val="15000"/>
               </a:schemeClr>
             </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>306546</xdr:colOff>
+      <xdr:row>105</xdr:row>
+      <xdr:rowOff>8964</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>247763</xdr:colOff>
+      <xdr:row>106</xdr:row>
+      <xdr:rowOff>181273</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="37" name="Rectangle 36">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D4583E2E-FFF3-28B5-39CE-1FD6E06A9061}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16156146" y="20054046"/>
+          <a:ext cx="550817" cy="365051"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="tx1"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1050">
+              <a:effectLst/>
+            </a:rPr>
+            <a:t>writer</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-DE" sz="1050">
+            <a:effectLst/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>306546</xdr:colOff>
+      <xdr:row>100</xdr:row>
+      <xdr:rowOff>163269</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>247763</xdr:colOff>
+      <xdr:row>102</xdr:row>
+      <xdr:rowOff>142837</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="38" name="Rectangle 37">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2BD66321-4727-684F-B34C-00FDDFE25BA1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16156146" y="19244645"/>
+          <a:ext cx="550817" cy="365051"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="tx1"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000">
+              <a:effectLst/>
+            </a:rPr>
+            <a:t>streamer</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-DE" sz="1000">
+            <a:effectLst/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>357436</xdr:colOff>
+      <xdr:row>85</xdr:row>
+      <xdr:rowOff>3794</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>300558</xdr:colOff>
+      <xdr:row>86</xdr:row>
+      <xdr:rowOff>173862</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="40" name="Rectangle 39">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{62AA6709-2187-4623-4F90-DD62F8F78338}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7063036" y="16196294"/>
+          <a:ext cx="552722" cy="360568"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="tx1"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1050">
+              <a:effectLst/>
+            </a:rPr>
+            <a:t>writer</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-DE" sz="1050">
+            <a:effectLst/>
           </a:endParaRPr>
         </a:p>
       </xdr:txBody>
@@ -19671,7 +19902,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AEB2071-28A2-48BB-B77C-31D6CC6F6BEA}">
-  <dimension ref="B2:AG111"/>
+  <dimension ref="B2:AG112"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="16384" width="9.140625" style="8"/>
@@ -22126,7 +22357,7 @@
       <c r="K88" s="13"/>
       <c r="L88" s="20"/>
       <c r="M88" s="13"/>
-      <c r="N88" s="17"/>
+      <c r="N88" s="9"/>
       <c r="O88" s="9"/>
       <c r="P88" s="21"/>
       <c r="Q88" s="12"/>
@@ -22160,7 +22391,7 @@
       <c r="K89" s="13"/>
       <c r="L89" s="20"/>
       <c r="M89" s="13"/>
-      <c r="N89" s="12"/>
+      <c r="N89" s="17"/>
       <c r="O89" s="9"/>
       <c r="P89" s="21"/>
       <c r="Q89" s="12"/>
@@ -22259,7 +22490,7 @@
       <c r="H92" s="13"/>
       <c r="I92" s="9"/>
       <c r="J92" s="21"/>
-      <c r="K92" s="17"/>
+      <c r="K92" s="13"/>
       <c r="L92" s="20"/>
       <c r="M92" s="13"/>
       <c r="N92" s="12"/>
@@ -22268,10 +22499,10 @@
       <c r="Q92" s="12"/>
       <c r="R92" s="9"/>
       <c r="S92" s="21"/>
-      <c r="T92" s="17"/>
+      <c r="T92" s="13"/>
       <c r="U92" s="20"/>
       <c r="V92" s="13"/>
-      <c r="W92" s="12"/>
+      <c r="W92" s="13"/>
       <c r="X92" s="9"/>
       <c r="Y92" s="21"/>
       <c r="Z92" s="13"/>
@@ -22336,9 +22567,7 @@
       <c r="Q94" s="12"/>
       <c r="R94" s="9"/>
       <c r="S94" s="21"/>
-      <c r="T94" s="17" t="s">
-        <v>72</v>
-      </c>
+      <c r="T94" s="17"/>
       <c r="U94" s="20"/>
       <c r="V94" s="13"/>
       <c r="W94" s="12"/>
@@ -22363,7 +22592,7 @@
       <c r="H95" s="13"/>
       <c r="I95" s="9"/>
       <c r="J95" s="21"/>
-      <c r="K95" s="13"/>
+      <c r="K95" s="17"/>
       <c r="L95" s="20"/>
       <c r="M95" s="13"/>
       <c r="N95" s="12"/>
@@ -22372,18 +22601,18 @@
       <c r="Q95" s="12"/>
       <c r="R95" s="9"/>
       <c r="S95" s="21"/>
-      <c r="T95" s="17"/>
+      <c r="T95" s="17" t="s">
+        <v>72</v>
+      </c>
       <c r="U95" s="20"/>
       <c r="V95" s="13"/>
-      <c r="W95" s="12" t="s">
-        <v>74</v>
-      </c>
+      <c r="W95" s="12"/>
       <c r="X95" s="9"/>
       <c r="Y95" s="21"/>
-      <c r="Z95" s="19"/>
+      <c r="Z95" s="13"/>
       <c r="AA95" s="20"/>
       <c r="AB95" s="13"/>
-      <c r="AC95" s="19"/>
+      <c r="AC95" s="13"/>
       <c r="AD95" s="20"/>
       <c r="AE95" s="13"/>
       <c r="AF95" s="9"/>
@@ -22412,7 +22641,7 @@
       <c r="U96" s="20"/>
       <c r="V96" s="13"/>
       <c r="W96" s="12" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="X96" s="9"/>
       <c r="Y96" s="21"/>
@@ -22447,13 +22676,15 @@
       <c r="T97" s="17"/>
       <c r="U97" s="20"/>
       <c r="V97" s="13"/>
-      <c r="W97" s="13"/>
+      <c r="W97" s="12" t="s">
+        <v>73</v>
+      </c>
       <c r="X97" s="9"/>
       <c r="Y97" s="21"/>
-      <c r="Z97" s="13"/>
+      <c r="Z97" s="19"/>
       <c r="AA97" s="20"/>
       <c r="AB97" s="13"/>
-      <c r="AC97" s="13"/>
+      <c r="AC97" s="19"/>
       <c r="AD97" s="20"/>
       <c r="AE97" s="13"/>
       <c r="AF97" s="9"/>
@@ -22506,13 +22737,13 @@
       <c r="K99" s="13"/>
       <c r="L99" s="20"/>
       <c r="M99" s="13"/>
-      <c r="N99" s="9"/>
+      <c r="N99" s="12"/>
       <c r="O99" s="9"/>
       <c r="P99" s="21"/>
-      <c r="Q99" s="9"/>
+      <c r="Q99" s="12"/>
       <c r="R99" s="9"/>
       <c r="S99" s="21"/>
-      <c r="T99" s="22"/>
+      <c r="T99" s="17"/>
       <c r="U99" s="20"/>
       <c r="V99" s="13"/>
       <c r="W99" s="13"/>
@@ -22521,9 +22752,7 @@
       <c r="Z99" s="13"/>
       <c r="AA99" s="20"/>
       <c r="AB99" s="13"/>
-      <c r="AC99" s="14" t="s">
-        <v>108</v>
-      </c>
+      <c r="AC99" s="13"/>
       <c r="AD99" s="20"/>
       <c r="AE99" s="13"/>
       <c r="AF99" s="9"/>
@@ -22557,7 +22786,7 @@
       <c r="Z100" s="13"/>
       <c r="AA100" s="20"/>
       <c r="AB100" s="13"/>
-      <c r="AC100" s="13"/>
+      <c r="AC100" s="14"/>
       <c r="AD100" s="20"/>
       <c r="AE100" s="13"/>
       <c r="AF100" s="9"/>
@@ -22591,7 +22820,9 @@
       <c r="Z101" s="13"/>
       <c r="AA101" s="20"/>
       <c r="AB101" s="13"/>
-      <c r="AC101" s="13"/>
+      <c r="AC101" s="14" t="s">
+        <v>108</v>
+      </c>
       <c r="AD101" s="20"/>
       <c r="AE101" s="13"/>
       <c r="AF101" s="9"/>
@@ -22644,7 +22875,7 @@
       <c r="K103" s="13"/>
       <c r="L103" s="20"/>
       <c r="M103" s="13"/>
-      <c r="N103" s="30"/>
+      <c r="N103" s="9"/>
       <c r="O103" s="9"/>
       <c r="P103" s="21"/>
       <c r="Q103" s="9"/>
@@ -22678,7 +22909,7 @@
       <c r="K104" s="13"/>
       <c r="L104" s="20"/>
       <c r="M104" s="13"/>
-      <c r="N104" s="11"/>
+      <c r="N104" s="30"/>
       <c r="O104" s="9"/>
       <c r="P104" s="21"/>
       <c r="Q104" s="9"/>
@@ -22746,7 +22977,7 @@
       <c r="K106" s="13"/>
       <c r="L106" s="20"/>
       <c r="M106" s="13"/>
-      <c r="N106" s="9"/>
+      <c r="N106" s="11"/>
       <c r="O106" s="9"/>
       <c r="P106" s="21"/>
       <c r="Q106" s="9"/>
@@ -22872,34 +23103,34 @@
     <row r="110" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B110" s="9"/>
       <c r="C110" s="9"/>
-      <c r="D110" s="9"/>
-      <c r="E110" s="9"/>
-      <c r="F110" s="9"/>
-      <c r="G110" s="9"/>
-      <c r="H110" s="9"/>
+      <c r="D110" s="21"/>
+      <c r="E110" s="13"/>
+      <c r="F110" s="20"/>
+      <c r="G110" s="13"/>
+      <c r="H110" s="13"/>
       <c r="I110" s="9"/>
-      <c r="J110" s="9"/>
-      <c r="K110" s="9"/>
-      <c r="L110" s="9"/>
-      <c r="M110" s="9"/>
+      <c r="J110" s="21"/>
+      <c r="K110" s="13"/>
+      <c r="L110" s="20"/>
+      <c r="M110" s="13"/>
       <c r="N110" s="9"/>
       <c r="O110" s="9"/>
-      <c r="P110" s="9"/>
+      <c r="P110" s="21"/>
       <c r="Q110" s="9"/>
       <c r="R110" s="9"/>
-      <c r="S110" s="9"/>
-      <c r="T110" s="9"/>
-      <c r="U110" s="9"/>
-      <c r="V110" s="9"/>
-      <c r="W110" s="9"/>
+      <c r="S110" s="21"/>
+      <c r="T110" s="22"/>
+      <c r="U110" s="20"/>
+      <c r="V110" s="13"/>
+      <c r="W110" s="13"/>
       <c r="X110" s="9"/>
-      <c r="Y110" s="9"/>
-      <c r="Z110" s="9"/>
-      <c r="AA110" s="9"/>
-      <c r="AB110" s="9"/>
-      <c r="AC110" s="9"/>
-      <c r="AD110" s="9"/>
-      <c r="AE110" s="9"/>
+      <c r="Y110" s="21"/>
+      <c r="Z110" s="13"/>
+      <c r="AA110" s="20"/>
+      <c r="AB110" s="13"/>
+      <c r="AC110" s="13"/>
+      <c r="AD110" s="20"/>
+      <c r="AE110" s="13"/>
       <c r="AF110" s="9"/>
       <c r="AG110" s="9"/>
     </row>
@@ -22936,6 +23167,40 @@
       <c r="AE111" s="9"/>
       <c r="AF111" s="9"/>
       <c r="AG111" s="9"/>
+    </row>
+    <row r="112" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="B112" s="9"/>
+      <c r="C112" s="9"/>
+      <c r="D112" s="9"/>
+      <c r="E112" s="9"/>
+      <c r="F112" s="9"/>
+      <c r="G112" s="9"/>
+      <c r="H112" s="9"/>
+      <c r="I112" s="9"/>
+      <c r="J112" s="9"/>
+      <c r="K112" s="9"/>
+      <c r="L112" s="9"/>
+      <c r="M112" s="9"/>
+      <c r="N112" s="9"/>
+      <c r="O112" s="9"/>
+      <c r="P112" s="9"/>
+      <c r="Q112" s="9"/>
+      <c r="R112" s="9"/>
+      <c r="S112" s="9"/>
+      <c r="T112" s="9"/>
+      <c r="U112" s="9"/>
+      <c r="V112" s="9"/>
+      <c r="W112" s="9"/>
+      <c r="X112" s="9"/>
+      <c r="Y112" s="9"/>
+      <c r="Z112" s="9"/>
+      <c r="AA112" s="9"/>
+      <c r="AB112" s="9"/>
+      <c r="AC112" s="9"/>
+      <c r="AD112" s="9"/>
+      <c r="AE112" s="9"/>
+      <c r="AF112" s="9"/>
+      <c r="AG112" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Docs updated - MQTT port 1883 vs 9001
</commit_message>
<xml_diff>
--- a/_concept_6G_integration/MCS_Fall_Detection.xlsx
+++ b/_concept_6G_integration/MCS_Fall_Detection.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hayat\Documents\6G\FallDetection_new\_concept_6G_integration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCA650CF-BBE3-4C6E-9889-3B62ACDAAACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AF15102-E15E-49E2-BA99-3255AC721A5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20544" yWindow="-2970" windowWidth="23232" windowHeight="13872" activeTab="3" xr2:uid="{55F2A534-9267-4FFE-9D89-C2FA8C43E60F}"/>
+    <workbookView xWindow="20544" yWindow="-2970" windowWidth="23232" windowHeight="13872" activeTab="2" xr2:uid="{55F2A534-9267-4FFE-9D89-C2FA8C43E60F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -4974,83 +4974,6 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>24</xdr:col>
-      <xdr:colOff>185539</xdr:colOff>
-      <xdr:row>49</xdr:row>
-      <xdr:rowOff>25053</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>26</xdr:col>
-      <xdr:colOff>4564</xdr:colOff>
-      <xdr:row>52</xdr:row>
-      <xdr:rowOff>101253</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="63" name="Rectangle 62">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4F1F71BB-239D-455A-9480-1D1B1E3D79F9}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="14815939" y="9953465"/>
-          <a:ext cx="1038225" cy="654423"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="bg1">
-            <a:lumMod val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="15000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-GB" sz="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>caregiver DB ??</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-DE" sz="1200">
-            <a:solidFill>
-              <a:schemeClr val="bg1"/>
-            </a:solidFill>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>24</xdr:col>
       <xdr:colOff>131717</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>151856</xdr:rowOff>
@@ -6093,6 +6016,17 @@
               </a:solidFill>
             </a:rPr>
             <a:t>MinIO</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1200">
+              <a:solidFill>
+                <a:srgbClr val="0070C0"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>:9002</a:t>
           </a:r>
           <a:endParaRPr lang="en-DE" sz="1200">
             <a:solidFill>
@@ -6825,16 +6759,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>98628</xdr:colOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>486554</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>55262</xdr:rowOff>
+      <xdr:rowOff>48335</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>517728</xdr:colOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>98886</xdr:colOff>
       <xdr:row>27</xdr:row>
-      <xdr:rowOff>133703</xdr:rowOff>
+      <xdr:rowOff>126776</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -6849,8 +6783,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10461828" y="5122562"/>
-          <a:ext cx="1028700" cy="649941"/>
+          <a:off x="10240154" y="5174517"/>
+          <a:ext cx="1441132" cy="660332"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6910,7 +6844,18 @@
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
             </a:rPr>
-            <a:t>:1883</a:t>
+            <a:t>:1883 (TCP)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>:9001 (Websocket)</a:t>
           </a:r>
           <a:endParaRPr lang="en-DE" sz="1200">
             <a:solidFill>
@@ -7955,6 +7900,204 @@
             <a:t>:8001</a:t>
           </a:r>
           <a:endParaRPr lang="en-DE" sz="1200">
+            <a:solidFill>
+              <a:schemeClr val="bg1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>148782</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>15292</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>578639</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>94956</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="23" name="Rectangle 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9E45DC88-B6F5-7A9D-898E-5CCA06D8FB11}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14779182" y="8438856"/>
+          <a:ext cx="1039457" cy="661555"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="002060"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:srgbClr val="002060"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1200">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Postgres</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>(fall</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> history)</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-DE" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="bg1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>148782</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>56856</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>580544</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>136520</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="24" name="Rectangle 23">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3F2AD9E9-A15A-91E2-E259-DCD22A781E72}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14779182" y="9838165"/>
+          <a:ext cx="1041362" cy="661555"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="002060"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:srgbClr val="002060"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1200">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Postgres</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>(ml_flow</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>)</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-DE" sz="1100">
             <a:solidFill>
               <a:schemeClr val="bg1"/>
             </a:solidFill>
@@ -19219,7 +19362,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8F5F8DD-066E-404B-880B-D3D7B4214C4F}">
-  <dimension ref="E3:AI49"/>
+  <dimension ref="E3:AI57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="27" max="27" width="4.7109375" customWidth="1"/>
@@ -19885,9 +20028,201 @@
     </row>
     <row r="44" spans="5:35" x14ac:dyDescent="0.25">
       <c r="E44" s="1"/>
-    </row>
-    <row r="49" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="X44" s="8"/>
+      <c r="Y44" s="8"/>
+      <c r="Z44" s="8"/>
+      <c r="AA44" s="8"/>
+      <c r="AB44" s="8"/>
+      <c r="AC44" s="8"/>
+      <c r="AD44" s="8"/>
+      <c r="AE44" s="8"/>
+      <c r="AF44" s="8"/>
+      <c r="AG44" s="8"/>
+      <c r="AH44" s="8"/>
+      <c r="AI44" s="8"/>
+    </row>
+    <row r="45" spans="5:35" x14ac:dyDescent="0.25">
+      <c r="X45" s="8"/>
+      <c r="Y45" s="8"/>
+      <c r="Z45" s="8"/>
+      <c r="AA45" s="8"/>
+      <c r="AB45" s="8"/>
+      <c r="AC45" s="8"/>
+      <c r="AD45" s="8"/>
+      <c r="AE45" s="8"/>
+      <c r="AF45" s="8"/>
+      <c r="AG45" s="8"/>
+      <c r="AH45" s="8"/>
+      <c r="AI45" s="8"/>
+    </row>
+    <row r="46" spans="5:35" x14ac:dyDescent="0.25">
+      <c r="X46" s="8"/>
+      <c r="Y46" s="8"/>
+      <c r="Z46" s="8"/>
+      <c r="AA46" s="8"/>
+      <c r="AB46" s="8"/>
+      <c r="AC46" s="8"/>
+      <c r="AD46" s="8"/>
+      <c r="AE46" s="8"/>
+      <c r="AF46" s="8"/>
+      <c r="AG46" s="8"/>
+      <c r="AH46" s="8"/>
+      <c r="AI46" s="8"/>
+    </row>
+    <row r="47" spans="5:35" x14ac:dyDescent="0.25">
+      <c r="X47" s="8"/>
+      <c r="Y47" s="8"/>
+      <c r="Z47" s="8"/>
+      <c r="AA47" s="8"/>
+      <c r="AB47" s="8"/>
+      <c r="AC47" s="8"/>
+      <c r="AD47" s="8"/>
+      <c r="AE47" s="8"/>
+      <c r="AF47" s="8"/>
+      <c r="AG47" s="8"/>
+      <c r="AH47" s="8"/>
+      <c r="AI47" s="8"/>
+    </row>
+    <row r="48" spans="5:35" x14ac:dyDescent="0.25">
+      <c r="X48" s="8"/>
+      <c r="Y48" s="8"/>
+      <c r="Z48" s="8"/>
+      <c r="AA48" s="8"/>
+      <c r="AB48" s="8"/>
+      <c r="AC48" s="8"/>
+      <c r="AD48" s="8"/>
+      <c r="AE48" s="8"/>
+      <c r="AF48" s="8"/>
+      <c r="AG48" s="8"/>
+      <c r="AH48" s="8"/>
+      <c r="AI48" s="8"/>
+    </row>
+    <row r="49" spans="5:35" x14ac:dyDescent="0.25">
       <c r="E49" s="1"/>
+      <c r="X49" s="8"/>
+      <c r="Y49" s="8"/>
+      <c r="Z49" s="8"/>
+      <c r="AA49" s="8"/>
+      <c r="AB49" s="8"/>
+      <c r="AC49" s="8"/>
+      <c r="AD49" s="8"/>
+      <c r="AE49" s="8"/>
+      <c r="AF49" s="8"/>
+      <c r="AG49" s="8"/>
+      <c r="AH49" s="8"/>
+      <c r="AI49" s="8"/>
+    </row>
+    <row r="50" spans="5:35" x14ac:dyDescent="0.25">
+      <c r="X50" s="8"/>
+      <c r="Y50" s="8"/>
+      <c r="Z50" s="8"/>
+      <c r="AA50" s="8"/>
+      <c r="AB50" s="8"/>
+      <c r="AC50" s="8"/>
+      <c r="AD50" s="8"/>
+      <c r="AE50" s="8"/>
+      <c r="AF50" s="8"/>
+      <c r="AG50" s="8"/>
+      <c r="AH50" s="8"/>
+      <c r="AI50" s="8"/>
+    </row>
+    <row r="51" spans="5:35" x14ac:dyDescent="0.25">
+      <c r="X51" s="8"/>
+      <c r="Y51" s="8"/>
+      <c r="Z51" s="8"/>
+      <c r="AA51" s="8"/>
+      <c r="AB51" s="8"/>
+      <c r="AC51" s="8"/>
+      <c r="AD51" s="8"/>
+      <c r="AE51" s="8"/>
+      <c r="AF51" s="8"/>
+      <c r="AG51" s="8"/>
+      <c r="AH51" s="8"/>
+      <c r="AI51" s="8"/>
+    </row>
+    <row r="52" spans="5:35" x14ac:dyDescent="0.25">
+      <c r="X52" s="8"/>
+      <c r="Y52" s="8"/>
+      <c r="Z52" s="8"/>
+      <c r="AA52" s="8"/>
+      <c r="AB52" s="8"/>
+      <c r="AC52" s="8"/>
+      <c r="AD52" s="8"/>
+      <c r="AE52" s="8"/>
+      <c r="AF52" s="8"/>
+      <c r="AG52" s="8"/>
+      <c r="AH52" s="8"/>
+      <c r="AI52" s="8"/>
+    </row>
+    <row r="53" spans="5:35" x14ac:dyDescent="0.25">
+      <c r="X53" s="8"/>
+      <c r="Y53" s="8"/>
+      <c r="Z53" s="8"/>
+      <c r="AA53" s="8"/>
+      <c r="AB53" s="8"/>
+      <c r="AC53" s="8"/>
+      <c r="AD53" s="8"/>
+      <c r="AE53" s="8"/>
+      <c r="AF53" s="8"/>
+      <c r="AG53" s="8"/>
+      <c r="AH53" s="8"/>
+      <c r="AI53" s="8"/>
+    </row>
+    <row r="54" spans="5:35" x14ac:dyDescent="0.25">
+      <c r="X54" s="8"/>
+      <c r="Y54" s="8"/>
+      <c r="Z54" s="8"/>
+      <c r="AA54" s="8"/>
+      <c r="AB54" s="8"/>
+      <c r="AC54" s="8"/>
+      <c r="AD54" s="8"/>
+      <c r="AE54" s="8"/>
+      <c r="AF54" s="8"/>
+      <c r="AG54" s="8"/>
+      <c r="AH54" s="8"/>
+      <c r="AI54" s="8"/>
+    </row>
+    <row r="55" spans="5:35" x14ac:dyDescent="0.25">
+      <c r="X55" s="8"/>
+      <c r="Y55" s="8"/>
+      <c r="Z55" s="8"/>
+      <c r="AA55" s="8"/>
+      <c r="AB55" s="8"/>
+      <c r="AC55" s="8"/>
+      <c r="AD55" s="8"/>
+      <c r="AE55" s="8"/>
+      <c r="AF55" s="8"/>
+      <c r="AG55" s="8"/>
+      <c r="AH55" s="8"/>
+      <c r="AI55" s="8"/>
+    </row>
+    <row r="56" spans="5:35" x14ac:dyDescent="0.25">
+      <c r="X56" s="8"/>
+      <c r="Y56" s="8"/>
+      <c r="Z56" s="8"/>
+      <c r="AA56" s="8"/>
+      <c r="AB56" s="8"/>
+      <c r="AC56" s="8"/>
+      <c r="AD56" s="8"/>
+      <c r="AE56" s="8"/>
+      <c r="AF56" s="8"/>
+      <c r="AG56" s="8"/>
+      <c r="AH56" s="8"/>
+      <c r="AI56" s="8"/>
+    </row>
+    <row r="57" spans="5:35" x14ac:dyDescent="0.25">
+      <c r="X57" s="8"/>
+      <c r="Y57" s="8"/>
+      <c r="Z57" s="8"/>
+      <c r="AA57" s="8"/>
+      <c r="AB57" s="8"/>
+      <c r="AC57" s="8"/>
+      <c r="AD57" s="8"/>
+      <c r="AE57" s="8"/>
+      <c r="AF57" s="8"/>
+      <c r="AG57" s="8"/>
+      <c r="AH57" s="8"/>
+      <c r="AI57" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
docs for handing over
</commit_message>
<xml_diff>
--- a/_concept_6G_integration/MCS_Fall_Detection.xlsx
+++ b/_concept_6G_integration/MCS_Fall_Detection.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hayat\Documents\6G\FallDetection_new\_concept_6G_integration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{862AC03C-A186-4933-89C3-6974FDE1CC87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC6342B6-B155-47D2-B439-00880B043E0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20544" yWindow="-2970" windowWidth="23232" windowHeight="13872" firstSheet="1" activeTab="2" xr2:uid="{55F2A534-9267-4FFE-9D89-C2FA8C43E60F}"/>
+    <workbookView xWindow="20544" yWindow="-2970" windowWidth="23232" windowHeight="13872" firstSheet="1" activeTab="4" xr2:uid="{55F2A534-9267-4FFE-9D89-C2FA8C43E60F}"/>
   </bookViews>
   <sheets>
     <sheet name="Architecture (2)" sheetId="7" state="hidden" r:id="rId1"/>
     <sheet name="Architecture" sheetId="3" r:id="rId2"/>
     <sheet name="SequenceDiagram" sheetId="4" r:id="rId3"/>
     <sheet name="Sheet1" sheetId="6" r:id="rId4"/>
-    <sheet name="SequenceDiagram (2)" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="info to share" sheetId="8" r:id="rId5"/>
+    <sheet name="SequenceDiagram (2)" sheetId="5" state="hidden" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="119">
   <si>
     <t xml:space="preserve">Additional Components </t>
   </si>
@@ -317,6 +318,102 @@
   <si>
     <t>fall_dashboard background task</t>
   </si>
+  <si>
+    <t>which images are custom or public, hence which needs to be pushed to public registry</t>
+  </si>
+  <si>
+    <t>Document</t>
+  </si>
+  <si>
+    <t xml:space="preserve">k8s </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient </t>
+  </si>
+  <si>
+    <t>Caregiver</t>
+  </si>
+  <si>
+    <t>Mobile app integration</t>
+  </si>
+  <si>
+    <t>web app integration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">which code/file is shared and which is not </t>
+  </si>
+  <si>
+    <t>Fall detection algorithm</t>
+  </si>
+  <si>
+    <t>Fall detection system</t>
+  </si>
+  <si>
+    <t xml:space="preserve">what is the data input and what is the model and what is the output </t>
+  </si>
+  <si>
+    <t>how it is trained</t>
+  </si>
+  <si>
+    <t>how to manage model version</t>
+  </si>
+  <si>
+    <t>user flow (patient)</t>
+  </si>
+  <si>
+    <t>user flow (caregiver)</t>
+  </si>
+  <si>
+    <t>user flow (admin/tech)</t>
+  </si>
+  <si>
+    <t>data contract (expected shape of data input and output)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prerequisite </t>
+  </si>
+  <si>
+    <t>what is missing pieces</t>
+  </si>
+  <si>
+    <t>what should happen</t>
+  </si>
+  <si>
+    <t>location of existing pieces and how to talk to each compnent</t>
+  </si>
+  <si>
+    <t>how to monitor its health and how/when to  retrain</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Admin user</t>
+  </si>
+  <si>
+    <t>link to user flow (patient)</t>
+  </si>
+  <si>
+    <t>link to user flow (caregiver)</t>
+  </si>
+  <si>
+    <t>link to user flow (admin/tech)</t>
+  </si>
+  <si>
+    <t>architrecture overview + sequence diagram</t>
+  </si>
+  <si>
+    <t>internal info</t>
+  </si>
+  <si>
+    <t xml:space="preserve">command list </t>
+  </si>
+  <si>
+    <t>override list</t>
+  </si>
+  <si>
+    <t>Step by step guide</t>
+  </si>
 </sst>
 </file>
 
@@ -440,7 +537,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -484,11 +581,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -537,11 +643,14 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -22009,15 +22118,15 @@
     </row>
     <row r="6" spans="18:35" ht="18.75" x14ac:dyDescent="0.3">
       <c r="X6" s="3"/>
-      <c r="Y6" s="26" t="s">
+      <c r="Y6" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="Z6" s="26"/>
-      <c r="AA6" s="26" t="s">
+      <c r="Z6" s="28"/>
+      <c r="AA6" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="AB6" s="26"/>
-      <c r="AC6" s="26"/>
+      <c r="AB6" s="28"/>
+      <c r="AC6" s="28"/>
       <c r="AD6" s="25"/>
       <c r="AE6" s="25"/>
       <c r="AF6" s="25"/>
@@ -22884,15 +22993,15 @@
     </row>
     <row r="6" spans="18:35" ht="18.75" x14ac:dyDescent="0.3">
       <c r="X6" s="3"/>
-      <c r="Y6" s="26" t="s">
+      <c r="Y6" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="Z6" s="26"/>
-      <c r="AA6" s="26" t="s">
+      <c r="Z6" s="28"/>
+      <c r="AA6" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="AB6" s="26"/>
-      <c r="AC6" s="26"/>
+      <c r="AB6" s="28"/>
+      <c r="AC6" s="28"/>
       <c r="AD6" s="20"/>
       <c r="AE6" s="20"/>
       <c r="AF6" s="20"/>
@@ -23062,14 +23171,14 @@
       <c r="Y16" s="3"/>
       <c r="Z16" s="3"/>
       <c r="AA16" s="3"/>
-      <c r="AB16" s="28" t="s">
+      <c r="AB16" s="27" t="s">
         <v>37</v>
       </c>
-      <c r="AC16" s="28"/>
-      <c r="AD16" s="28"/>
-      <c r="AE16" s="28"/>
-      <c r="AF16" s="28"/>
-      <c r="AG16" s="28" t="s">
+      <c r="AC16" s="27"/>
+      <c r="AD16" s="27"/>
+      <c r="AE16" s="27"/>
+      <c r="AF16" s="27"/>
+      <c r="AG16" s="27" t="s">
         <v>49</v>
       </c>
       <c r="AH16" s="3"/>
@@ -23080,14 +23189,14 @@
       <c r="Y17" s="3"/>
       <c r="Z17" s="3"/>
       <c r="AA17" s="3"/>
-      <c r="AB17" s="28" t="s">
+      <c r="AB17" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="AC17" s="28"/>
-      <c r="AD17" s="28"/>
-      <c r="AE17" s="28"/>
-      <c r="AF17" s="28"/>
-      <c r="AG17" s="28" t="s">
+      <c r="AC17" s="27"/>
+      <c r="AD17" s="27"/>
+      <c r="AE17" s="27"/>
+      <c r="AF17" s="27"/>
+      <c r="AG17" s="27" t="s">
         <v>48</v>
       </c>
       <c r="AH17" s="3"/>
@@ -23098,14 +23207,14 @@
       <c r="Y18" s="3"/>
       <c r="Z18" s="3"/>
       <c r="AA18" s="3"/>
-      <c r="AB18" s="28" t="s">
+      <c r="AB18" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="AC18" s="28"/>
-      <c r="AD18" s="28"/>
-      <c r="AE18" s="28"/>
-      <c r="AF18" s="28"/>
-      <c r="AG18" s="28" t="s">
+      <c r="AC18" s="27"/>
+      <c r="AD18" s="27"/>
+      <c r="AE18" s="27"/>
+      <c r="AF18" s="27"/>
+      <c r="AG18" s="27" t="s">
         <v>48</v>
       </c>
       <c r="AH18" s="3"/>
@@ -23257,7 +23366,7 @@
       <c r="AD28" s="3"/>
       <c r="AE28" s="3"/>
       <c r="AF28" s="3"/>
-      <c r="AG28" s="27" t="s">
+      <c r="AG28" s="26" t="s">
         <v>84</v>
       </c>
       <c r="AH28" s="3"/>
@@ -23275,7 +23384,7 @@
       <c r="AD29" s="3"/>
       <c r="AE29" s="3"/>
       <c r="AF29" s="3"/>
-      <c r="AG29" s="27" t="s">
+      <c r="AG29" s="26" t="s">
         <v>84</v>
       </c>
       <c r="AH29" s="3"/>
@@ -23293,7 +23402,7 @@
       <c r="AD30" s="3"/>
       <c r="AE30" s="3"/>
       <c r="AF30" s="3"/>
-      <c r="AG30" s="27" t="s">
+      <c r="AG30" s="26" t="s">
         <v>84</v>
       </c>
       <c r="AH30" s="3"/>
@@ -23311,7 +23420,7 @@
       <c r="AD31" s="3"/>
       <c r="AE31" s="3"/>
       <c r="AF31" s="3"/>
-      <c r="AG31" s="27" t="s">
+      <c r="AG31" s="26" t="s">
         <v>84</v>
       </c>
       <c r="AH31" s="3"/>
@@ -23329,7 +23438,7 @@
       <c r="AD32" s="3"/>
       <c r="AE32" s="3"/>
       <c r="AF32" s="3"/>
-      <c r="AG32" s="27" t="s">
+      <c r="AG32" s="26" t="s">
         <v>84</v>
       </c>
       <c r="AH32" s="3"/>
@@ -27272,6 +27381,185 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4BFEE13-EE03-4A51-A59E-ED03788FB866}">
+  <dimension ref="A2:C52"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="23.140625" customWidth="1"/>
+    <col min="2" max="2" width="78.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" s="29" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C6" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>95</v>
+      </c>
+      <c r="B11" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>96</v>
+      </c>
+      <c r="B17" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>92</v>
+      </c>
+      <c r="B24" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>93</v>
+      </c>
+      <c r="B30" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B31" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B32" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B33" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>90</v>
+      </c>
+      <c r="B40" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>91</v>
+      </c>
+      <c r="B46" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>110</v>
+      </c>
+      <c r="B52" t="s">
+        <v>102</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BD0ABB0-740C-45D8-A980-F8FD0FB04F00}">
   <dimension ref="B2:AA107"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>